<commit_message>
updating lending files to 1.0.2 with test result for all the tests.
Signed-off-by: mathurrohit875 <mathurrohit875@gmail.com>
</commit_message>
<xml_diff>
--- a/src/main/java/data/LendingData.xlsx
+++ b/src/main/java/data/LendingData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit.mathur\ChainProject\ChainTestProject\src\main\java\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6438813B-B385-4186-9A1E-2F3017817AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2E2506-0499-48A9-8018-8C0EC48DEF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="94">
   <si>
     <t>Type</t>
   </si>
@@ -307,19 +307,10 @@
     <t>cussdvioy</t>
   </si>
   <si>
-    <t>CSP186606</t>
-  </si>
-  <si>
-    <t>CSP186625</t>
-  </si>
-  <si>
-    <t>CSP186834</t>
-  </si>
-  <si>
-    <t>CSP186912</t>
-  </si>
-  <si>
-    <t>CSP200048</t>
+    <t>CSP250595</t>
+  </si>
+  <si>
+    <t>CSP212746</t>
   </si>
 </sst>
 </file>
@@ -982,7 +973,7 @@
         <v>80</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
@@ -990,7 +981,7 @@
         <v>81</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1348,7 +1339,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1364,7 +1355,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1713,7 +1704,7 @@
         <v>86</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -1887,7 +1878,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1903,7 +1894,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updating loan results new
Signed-off-by: mathurrohit875 <mathurrohit875@gmail.com>
</commit_message>
<xml_diff>
--- a/src/main/java/data/LendingData.xlsx
+++ b/src/main/java/data/LendingData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit.mathur\ChainProject\ChainTestProject\src\main\java\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E959FA4E-2644-40A4-8016-83971E405013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A5DAB0-76C0-4743-8E07-F41AEEE522EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="93">
   <si>
     <t>Type</t>
   </si>
@@ -307,19 +307,7 @@
     <t>cussdvioy</t>
   </si>
   <si>
-    <t>CSP207365</t>
-  </si>
-  <si>
     <t>CSP207493</t>
-  </si>
-  <si>
-    <t>CSP207517</t>
-  </si>
-  <si>
-    <t>CSP207567</t>
-  </si>
-  <si>
-    <t>CSP207843</t>
   </si>
 </sst>
 </file>
@@ -1142,7 +1130,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1158,7 +1146,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1348,7 +1336,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1364,7 +1352,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1713,7 +1701,7 @@
         <v>86</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -1887,7 +1875,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1903,7 +1891,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updating loan files with results and changes in pom file
Signed-off-by: mathurrohit875 <mathurrohit875@gmail.com>
</commit_message>
<xml_diff>
--- a/src/main/java/data/LendingData.xlsx
+++ b/src/main/java/data/LendingData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit.mathur\ChainProject\ChainTestProject\src\main\java\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A5DAB0-76C0-4743-8E07-F41AEEE522EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF724AF5-18F2-4B6F-A003-AF53C47BEEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoanDetail" sheetId="1" r:id="rId1"/>
+    <sheet name="LongTermLoan" sheetId="1" r:id="rId1"/>
     <sheet name="WeekendLoan" sheetId="2" r:id="rId2"/>
     <sheet name="ShortTermLoan" sheetId="3" r:id="rId3"/>
     <sheet name="OtherProductLoan" sheetId="4" r:id="rId4"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="95">
   <si>
     <t>Type</t>
   </si>
@@ -307,7 +307,13 @@
     <t>cussdvioy</t>
   </si>
   <si>
-    <t>CSP207493</t>
+    <t>Approval Email Doc</t>
+  </si>
+  <si>
+    <t>C:\\Users\\rohit.mathur\\Downloads\\431742525.pdf</t>
+  </si>
+  <si>
+    <t>CSP176984</t>
   </si>
 </sst>
 </file>
@@ -662,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="69.7265625" customWidth="1"/>
@@ -970,7 +976,7 @@
         <v>80</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
@@ -978,7 +984,15 @@
         <v>81</v>
       </c>
       <c r="B39" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>92</v>
+      </c>
+      <c r="B40" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -989,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05E87538-8091-4D89-92F7-1A5318D4CDAF}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" customWidth="1"/>
@@ -1130,7 +1144,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1146,7 +1160,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1186,6 +1200,14 @@
       </c>
       <c r="B25">
         <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1196,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CE6B162-CF77-4DEF-A251-D4C4731E90C4}">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" bestFit="1" customWidth="1"/>
@@ -1336,7 +1358,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1352,7 +1374,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1408,6 +1430,14 @@
       </c>
       <c r="B27">
         <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1417,7 +1447,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEAA7BCB-65AD-4776-B743-29A58193C791}">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="39.81640625" bestFit="1" customWidth="1"/>
@@ -1701,7 +1731,7 @@
         <v>86</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -1726,6 +1756,14 @@
       </c>
       <c r="B38" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1875,7 +1913,7 @@
         <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1891,7 +1929,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1931,6 +1969,14 @@
       </c>
       <c r="B25">
         <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Force Pass and Fail files updated
Signed-off-by: mathurrohit875 <mathurrohit875@gmail.com>
</commit_message>
<xml_diff>
--- a/src/main/java/data/LendingData.xlsx
+++ b/src/main/java/data/LendingData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit.mathur\ChainProject\ChainTestProject\src\main\java\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF724AF5-18F2-4B6F-A003-AF53C47BEEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D4D5DB-5447-4166-916E-7A7909103895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,7 +313,7 @@
     <t>C:\\Users\\rohit.mathur\\Downloads\\431742525.pdf</t>
   </si>
   <si>
-    <t>CSP176984</t>
+    <t>CSP178923</t>
   </si>
 </sst>
 </file>

</xml_diff>